<commit_message>
checks on sulfide sulfate capacity from GW26
</commit_message>
<xml_diff>
--- a/docs/benchmarking/materials-from-original-papers/Gorojovsky26.xlsx
+++ b/docs/benchmarking/materials-from-original-papers/Gorojovsky26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\erych\projects\VolFe\docs\benchmarking\materials-from-original-papers\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveuclac-my.sharepoint.com/personal/ucfbugh_ucl_ac_uk/Documents/Documents/research/degassing/volfe/2026-08-05 files not pushed to GitHub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04DB6947-B018-49B8-BAC0-43861081390A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{D0DBDB6B-7336-4609-93F0-9775D8AFD14D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A89FFF6-68C0-4162-855F-2CFCA47579B6}"/>
   <bookViews>
-    <workbookView xWindow="-4995" yWindow="-21720" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{32DF9F16-F33B-8948-9851-681D5E8C3787}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{32DF9F16-F33B-8948-9851-681D5E8C3787}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -2755,6 +2755,57 @@
     <xf numFmtId="2" fontId="9" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2762,6 +2813,33 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="10" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="21" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="18" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="10" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2787,14 +2865,8 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2808,14 +2880,8 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="18" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2841,82 +2907,16 @@
     <xf numFmtId="0" fontId="14" fillId="7" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="3" borderId="17" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="20" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="21" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="14" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="5" borderId="18" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="16" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -7860,25 +7860,24 @@
     <col min="7" max="8" width="10" style="2" customWidth="1"/>
     <col min="9" max="18" width="10.1640625" style="2" customWidth="1"/>
     <col min="19" max="21" width="10.5" style="2" customWidth="1"/>
-    <col min="22" max="22" width="11.5" style="2" customWidth="1"/>
-    <col min="23" max="131" width="11.5" style="2" hidden="1" customWidth="1"/>
-    <col min="132" max="134" width="14.5" style="2" hidden="1" customWidth="1"/>
-    <col min="135" max="135" width="11.5" style="2" hidden="1" customWidth="1"/>
-    <col min="136" max="144" width="14.5" style="2" hidden="1" customWidth="1"/>
-    <col min="145" max="145" width="11.5" style="2" hidden="1" customWidth="1"/>
-    <col min="146" max="148" width="14.5" style="2" hidden="1" customWidth="1"/>
-    <col min="149" max="149" width="11.5" style="2" hidden="1" customWidth="1"/>
-    <col min="150" max="151" width="14.5" style="2" hidden="1" customWidth="1"/>
-    <col min="152" max="152" width="11.5" style="2" hidden="1" customWidth="1"/>
-    <col min="153" max="153" width="14.5" style="2" hidden="1" customWidth="1"/>
-    <col min="154" max="161" width="11.5" style="2" hidden="1" customWidth="1"/>
-    <col min="162" max="166" width="14.5" style="2" hidden="1" customWidth="1"/>
-    <col min="167" max="167" width="11.5" style="2" hidden="1" customWidth="1"/>
-    <col min="168" max="170" width="16.83203125" style="2" hidden="1" customWidth="1"/>
-    <col min="171" max="172" width="14.5" style="2" hidden="1" customWidth="1"/>
-    <col min="173" max="173" width="13.33203125" style="2" hidden="1" customWidth="1"/>
-    <col min="174" max="174" width="11.5" style="2" hidden="1" customWidth="1"/>
-    <col min="175" max="177" width="14.5" style="2" hidden="1" customWidth="1"/>
+    <col min="22" max="131" width="11.5" style="2" customWidth="1"/>
+    <col min="132" max="134" width="14.5" style="2" customWidth="1"/>
+    <col min="135" max="135" width="11.5" style="2" customWidth="1"/>
+    <col min="136" max="144" width="14.5" style="2" customWidth="1"/>
+    <col min="145" max="145" width="11.5" style="2" customWidth="1"/>
+    <col min="146" max="148" width="14.5" style="2" customWidth="1"/>
+    <col min="149" max="149" width="11.5" style="2" customWidth="1"/>
+    <col min="150" max="151" width="14.5" style="2" customWidth="1"/>
+    <col min="152" max="152" width="11.5" style="2" customWidth="1"/>
+    <col min="153" max="153" width="14.5" style="2" customWidth="1"/>
+    <col min="154" max="161" width="11.5" style="2" customWidth="1"/>
+    <col min="162" max="166" width="14.5" style="2" customWidth="1"/>
+    <col min="167" max="167" width="11.5" style="2" customWidth="1"/>
+    <col min="168" max="170" width="16.83203125" style="2" customWidth="1"/>
+    <col min="171" max="172" width="14.5" style="2" customWidth="1"/>
+    <col min="173" max="173" width="13.33203125" style="2" customWidth="1"/>
+    <col min="174" max="174" width="11.5" style="2" customWidth="1"/>
+    <col min="175" max="177" width="14.5" style="2" customWidth="1"/>
     <col min="178" max="178" width="10.33203125" style="2" customWidth="1"/>
     <col min="179" max="179" width="13" style="2" customWidth="1"/>
     <col min="180" max="184" width="14.5" style="2" customWidth="1"/>
@@ -8112,167 +8111,167 @@
       <c r="R2" s="34"/>
       <c r="S2" s="34"/>
       <c r="T2" s="3"/>
-      <c r="U2" s="156" t="s">
+      <c r="U2" s="131" t="s">
         <v>2</v>
       </c>
-      <c r="V2" s="157"/>
-      <c r="W2" s="157"/>
-      <c r="X2" s="157"/>
-      <c r="Y2" s="157"/>
-      <c r="Z2" s="157"/>
-      <c r="AA2" s="157"/>
-      <c r="AB2" s="157"/>
-      <c r="AC2" s="157"/>
-      <c r="AD2" s="157"/>
-      <c r="AE2" s="157"/>
-      <c r="AF2" s="157"/>
-      <c r="AG2" s="157"/>
-      <c r="AH2" s="157"/>
-      <c r="AI2" s="157"/>
-      <c r="AJ2" s="157"/>
-      <c r="AK2" s="157"/>
-      <c r="AL2" s="157"/>
-      <c r="AM2" s="157"/>
-      <c r="AN2" s="157"/>
-      <c r="AO2" s="157"/>
-      <c r="AP2" s="157"/>
-      <c r="AQ2" s="157"/>
-      <c r="AR2" s="157"/>
-      <c r="AS2" s="157"/>
-      <c r="AT2" s="157"/>
-      <c r="AU2" s="157"/>
-      <c r="AV2" s="157"/>
-      <c r="AW2" s="157"/>
-      <c r="AX2" s="157"/>
-      <c r="AY2" s="157"/>
-      <c r="AZ2" s="157"/>
-      <c r="BA2" s="157"/>
-      <c r="BB2" s="157"/>
-      <c r="BC2" s="157"/>
-      <c r="BD2" s="157"/>
-      <c r="BE2" s="157"/>
-      <c r="BF2" s="157"/>
-      <c r="BG2" s="157"/>
-      <c r="BH2" s="157"/>
-      <c r="BI2" s="157"/>
-      <c r="BJ2" s="157"/>
-      <c r="BK2" s="157"/>
-      <c r="BL2" s="157"/>
-      <c r="BM2" s="157"/>
-      <c r="BN2" s="157"/>
-      <c r="BO2" s="157"/>
-      <c r="BP2" s="157"/>
-      <c r="BQ2" s="157"/>
-      <c r="BR2" s="157"/>
-      <c r="BS2" s="157"/>
-      <c r="BT2" s="157"/>
-      <c r="BU2" s="157"/>
-      <c r="BV2" s="157"/>
-      <c r="BW2" s="157"/>
-      <c r="BX2" s="157"/>
-      <c r="BY2" s="157"/>
-      <c r="BZ2" s="157"/>
-      <c r="CA2" s="157"/>
-      <c r="CB2" s="157"/>
-      <c r="CC2" s="157"/>
-      <c r="CD2" s="157"/>
-      <c r="CE2" s="157"/>
-      <c r="CF2" s="157"/>
-      <c r="CG2" s="157"/>
-      <c r="CH2" s="157"/>
-      <c r="CI2" s="157"/>
-      <c r="CJ2" s="157"/>
-      <c r="CK2" s="157"/>
-      <c r="CL2" s="157"/>
-      <c r="CM2" s="157"/>
-      <c r="CN2" s="157"/>
-      <c r="CO2" s="157"/>
-      <c r="CP2" s="157"/>
-      <c r="CQ2" s="157"/>
-      <c r="CR2" s="157"/>
-      <c r="CS2" s="157"/>
-      <c r="CT2" s="157"/>
-      <c r="CU2" s="157"/>
-      <c r="CV2" s="157"/>
-      <c r="CW2" s="157"/>
-      <c r="CX2" s="157"/>
-      <c r="CY2" s="157"/>
-      <c r="CZ2" s="157"/>
-      <c r="DA2" s="157"/>
-      <c r="DB2" s="157"/>
-      <c r="DC2" s="157"/>
-      <c r="DD2" s="157"/>
-      <c r="DE2" s="157"/>
-      <c r="DF2" s="157"/>
-      <c r="DG2" s="157"/>
-      <c r="DH2" s="157"/>
-      <c r="DI2" s="157"/>
-      <c r="DJ2" s="157"/>
-      <c r="DK2" s="157"/>
-      <c r="DL2" s="157"/>
-      <c r="DM2" s="157"/>
-      <c r="DN2" s="157"/>
-      <c r="DO2" s="157"/>
-      <c r="DP2" s="157"/>
-      <c r="DQ2" s="157"/>
-      <c r="DR2" s="157"/>
-      <c r="DS2" s="157"/>
-      <c r="DT2" s="157"/>
-      <c r="DU2" s="157"/>
-      <c r="DV2" s="157"/>
-      <c r="DW2" s="157"/>
-      <c r="DX2" s="157"/>
-      <c r="DY2" s="157"/>
-      <c r="DZ2" s="157"/>
-      <c r="EA2" s="157"/>
-      <c r="EB2" s="157"/>
-      <c r="EC2" s="157"/>
-      <c r="ED2" s="157"/>
-      <c r="EE2" s="157"/>
-      <c r="EF2" s="157"/>
-      <c r="EG2" s="157"/>
-      <c r="EH2" s="157"/>
-      <c r="EI2" s="157"/>
-      <c r="EJ2" s="157"/>
-      <c r="EK2" s="157"/>
-      <c r="EL2" s="157"/>
-      <c r="EM2" s="157"/>
-      <c r="EN2" s="157"/>
-      <c r="EO2" s="157"/>
-      <c r="EP2" s="157"/>
-      <c r="EQ2" s="157"/>
-      <c r="ER2" s="157"/>
-      <c r="ES2" s="157"/>
-      <c r="ET2" s="157"/>
-      <c r="EU2" s="157"/>
-      <c r="EV2" s="157"/>
-      <c r="EW2" s="157"/>
-      <c r="EX2" s="157"/>
-      <c r="EY2" s="157"/>
-      <c r="EZ2" s="157"/>
-      <c r="FA2" s="157"/>
-      <c r="FB2" s="157"/>
-      <c r="FC2" s="157"/>
-      <c r="FD2" s="157"/>
-      <c r="FE2" s="157"/>
-      <c r="FF2" s="157"/>
-      <c r="FG2" s="157"/>
-      <c r="FH2" s="157"/>
-      <c r="FI2" s="157"/>
-      <c r="FJ2" s="157"/>
-      <c r="FK2" s="157"/>
-      <c r="FL2" s="157"/>
-      <c r="FM2" s="157"/>
-      <c r="FN2" s="157"/>
-      <c r="FO2" s="157"/>
-      <c r="FP2" s="157"/>
-      <c r="FQ2" s="157"/>
-      <c r="FR2" s="157"/>
-      <c r="FS2" s="157"/>
-      <c r="FT2" s="157"/>
-      <c r="FU2" s="157"/>
-      <c r="FV2" s="157"/>
-      <c r="FW2" s="158"/>
+      <c r="V2" s="132"/>
+      <c r="W2" s="132"/>
+      <c r="X2" s="132"/>
+      <c r="Y2" s="132"/>
+      <c r="Z2" s="132"/>
+      <c r="AA2" s="132"/>
+      <c r="AB2" s="132"/>
+      <c r="AC2" s="132"/>
+      <c r="AD2" s="132"/>
+      <c r="AE2" s="132"/>
+      <c r="AF2" s="132"/>
+      <c r="AG2" s="132"/>
+      <c r="AH2" s="132"/>
+      <c r="AI2" s="132"/>
+      <c r="AJ2" s="132"/>
+      <c r="AK2" s="132"/>
+      <c r="AL2" s="132"/>
+      <c r="AM2" s="132"/>
+      <c r="AN2" s="132"/>
+      <c r="AO2" s="132"/>
+      <c r="AP2" s="132"/>
+      <c r="AQ2" s="132"/>
+      <c r="AR2" s="132"/>
+      <c r="AS2" s="132"/>
+      <c r="AT2" s="132"/>
+      <c r="AU2" s="132"/>
+      <c r="AV2" s="132"/>
+      <c r="AW2" s="132"/>
+      <c r="AX2" s="132"/>
+      <c r="AY2" s="132"/>
+      <c r="AZ2" s="132"/>
+      <c r="BA2" s="132"/>
+      <c r="BB2" s="132"/>
+      <c r="BC2" s="132"/>
+      <c r="BD2" s="132"/>
+      <c r="BE2" s="132"/>
+      <c r="BF2" s="132"/>
+      <c r="BG2" s="132"/>
+      <c r="BH2" s="132"/>
+      <c r="BI2" s="132"/>
+      <c r="BJ2" s="132"/>
+      <c r="BK2" s="132"/>
+      <c r="BL2" s="132"/>
+      <c r="BM2" s="132"/>
+      <c r="BN2" s="132"/>
+      <c r="BO2" s="132"/>
+      <c r="BP2" s="132"/>
+      <c r="BQ2" s="132"/>
+      <c r="BR2" s="132"/>
+      <c r="BS2" s="132"/>
+      <c r="BT2" s="132"/>
+      <c r="BU2" s="132"/>
+      <c r="BV2" s="132"/>
+      <c r="BW2" s="132"/>
+      <c r="BX2" s="132"/>
+      <c r="BY2" s="132"/>
+      <c r="BZ2" s="132"/>
+      <c r="CA2" s="132"/>
+      <c r="CB2" s="132"/>
+      <c r="CC2" s="132"/>
+      <c r="CD2" s="132"/>
+      <c r="CE2" s="132"/>
+      <c r="CF2" s="132"/>
+      <c r="CG2" s="132"/>
+      <c r="CH2" s="132"/>
+      <c r="CI2" s="132"/>
+      <c r="CJ2" s="132"/>
+      <c r="CK2" s="132"/>
+      <c r="CL2" s="132"/>
+      <c r="CM2" s="132"/>
+      <c r="CN2" s="132"/>
+      <c r="CO2" s="132"/>
+      <c r="CP2" s="132"/>
+      <c r="CQ2" s="132"/>
+      <c r="CR2" s="132"/>
+      <c r="CS2" s="132"/>
+      <c r="CT2" s="132"/>
+      <c r="CU2" s="132"/>
+      <c r="CV2" s="132"/>
+      <c r="CW2" s="132"/>
+      <c r="CX2" s="132"/>
+      <c r="CY2" s="132"/>
+      <c r="CZ2" s="132"/>
+      <c r="DA2" s="132"/>
+      <c r="DB2" s="132"/>
+      <c r="DC2" s="132"/>
+      <c r="DD2" s="132"/>
+      <c r="DE2" s="132"/>
+      <c r="DF2" s="132"/>
+      <c r="DG2" s="132"/>
+      <c r="DH2" s="132"/>
+      <c r="DI2" s="132"/>
+      <c r="DJ2" s="132"/>
+      <c r="DK2" s="132"/>
+      <c r="DL2" s="132"/>
+      <c r="DM2" s="132"/>
+      <c r="DN2" s="132"/>
+      <c r="DO2" s="132"/>
+      <c r="DP2" s="132"/>
+      <c r="DQ2" s="132"/>
+      <c r="DR2" s="132"/>
+      <c r="DS2" s="132"/>
+      <c r="DT2" s="132"/>
+      <c r="DU2" s="132"/>
+      <c r="DV2" s="132"/>
+      <c r="DW2" s="132"/>
+      <c r="DX2" s="132"/>
+      <c r="DY2" s="132"/>
+      <c r="DZ2" s="132"/>
+      <c r="EA2" s="132"/>
+      <c r="EB2" s="132"/>
+      <c r="EC2" s="132"/>
+      <c r="ED2" s="132"/>
+      <c r="EE2" s="132"/>
+      <c r="EF2" s="132"/>
+      <c r="EG2" s="132"/>
+      <c r="EH2" s="132"/>
+      <c r="EI2" s="132"/>
+      <c r="EJ2" s="132"/>
+      <c r="EK2" s="132"/>
+      <c r="EL2" s="132"/>
+      <c r="EM2" s="132"/>
+      <c r="EN2" s="132"/>
+      <c r="EO2" s="132"/>
+      <c r="EP2" s="132"/>
+      <c r="EQ2" s="132"/>
+      <c r="ER2" s="132"/>
+      <c r="ES2" s="132"/>
+      <c r="ET2" s="132"/>
+      <c r="EU2" s="132"/>
+      <c r="EV2" s="132"/>
+      <c r="EW2" s="132"/>
+      <c r="EX2" s="132"/>
+      <c r="EY2" s="132"/>
+      <c r="EZ2" s="132"/>
+      <c r="FA2" s="132"/>
+      <c r="FB2" s="132"/>
+      <c r="FC2" s="132"/>
+      <c r="FD2" s="132"/>
+      <c r="FE2" s="132"/>
+      <c r="FF2" s="132"/>
+      <c r="FG2" s="132"/>
+      <c r="FH2" s="132"/>
+      <c r="FI2" s="132"/>
+      <c r="FJ2" s="132"/>
+      <c r="FK2" s="132"/>
+      <c r="FL2" s="132"/>
+      <c r="FM2" s="132"/>
+      <c r="FN2" s="132"/>
+      <c r="FO2" s="132"/>
+      <c r="FP2" s="132"/>
+      <c r="FQ2" s="132"/>
+      <c r="FR2" s="132"/>
+      <c r="FS2" s="132"/>
+      <c r="FT2" s="132"/>
+      <c r="FU2" s="132"/>
+      <c r="FV2" s="132"/>
+      <c r="FW2" s="133"/>
       <c r="FX2" s="1"/>
       <c r="FY2" s="1"/>
       <c r="FZ2" s="1"/>
@@ -8883,24 +8882,24 @@
       <c r="C6" s="21"/>
       <c r="D6" s="34"/>
       <c r="E6" s="34"/>
-      <c r="F6" s="127" t="s">
+      <c r="F6" s="153" t="s">
         <v>5</v>
       </c>
-      <c r="G6" s="128"/>
-      <c r="H6" s="128"/>
-      <c r="I6" s="128"/>
-      <c r="J6" s="128"/>
-      <c r="K6" s="128"/>
-      <c r="L6" s="128"/>
-      <c r="M6" s="128"/>
-      <c r="N6" s="128"/>
-      <c r="O6" s="128"/>
-      <c r="P6" s="128"/>
-      <c r="Q6" s="128"/>
-      <c r="R6" s="128"/>
-      <c r="S6" s="128"/>
-      <c r="T6" s="128"/>
-      <c r="U6" s="129"/>
+      <c r="G6" s="154"/>
+      <c r="H6" s="154"/>
+      <c r="I6" s="154"/>
+      <c r="J6" s="154"/>
+      <c r="K6" s="154"/>
+      <c r="L6" s="154"/>
+      <c r="M6" s="154"/>
+      <c r="N6" s="154"/>
+      <c r="O6" s="154"/>
+      <c r="P6" s="154"/>
+      <c r="Q6" s="154"/>
+      <c r="R6" s="154"/>
+      <c r="S6" s="154"/>
+      <c r="T6" s="154"/>
+      <c r="U6" s="155"/>
       <c r="V6" s="3"/>
       <c r="W6" s="34"/>
       <c r="X6" s="34"/>
@@ -9015,95 +9014,95 @@
       <c r="EC6" s="34"/>
       <c r="ED6" s="34"/>
       <c r="EE6" s="34"/>
-      <c r="EF6" s="133" t="s">
+      <c r="EF6" s="144" t="s">
         <v>6</v>
       </c>
-      <c r="EG6" s="134"/>
-      <c r="EH6" s="134"/>
+      <c r="EG6" s="159"/>
+      <c r="EH6" s="159"/>
       <c r="EI6" s="135"/>
       <c r="EJ6" s="34"/>
-      <c r="EK6" s="139" t="s">
+      <c r="EK6" s="163" t="s">
         <v>7</v>
       </c>
-      <c r="EL6" s="140"/>
-      <c r="EM6" s="140"/>
-      <c r="EN6" s="140"/>
-      <c r="EO6" s="140"/>
-      <c r="EP6" s="140"/>
-      <c r="EQ6" s="143" t="s">
+      <c r="EL6" s="134"/>
+      <c r="EM6" s="134"/>
+      <c r="EN6" s="134"/>
+      <c r="EO6" s="134"/>
+      <c r="EP6" s="134"/>
+      <c r="EQ6" s="165" t="s">
         <v>8</v>
       </c>
-      <c r="ER6" s="144"/>
-      <c r="ES6" s="145"/>
+      <c r="ER6" s="166"/>
+      <c r="ES6" s="167"/>
       <c r="ET6" s="71"/>
-      <c r="EU6" s="149" t="s">
+      <c r="EU6" s="171" t="s">
         <v>9</v>
       </c>
       <c r="EV6" s="135"/>
       <c r="EW6" s="71"/>
-      <c r="EX6" s="152" t="s">
+      <c r="EX6" s="127" t="s">
         <v>10</v>
       </c>
       <c r="EY6" s="71"/>
-      <c r="EZ6" s="154" t="s">
+      <c r="EZ6" s="173" t="s">
         <v>11</v>
       </c>
-      <c r="FA6" s="140"/>
-      <c r="FB6" s="140"/>
-      <c r="FC6" s="140"/>
+      <c r="FA6" s="134"/>
+      <c r="FB6" s="134"/>
+      <c r="FC6" s="134"/>
       <c r="FD6" s="135"/>
       <c r="FE6" s="71"/>
-      <c r="FF6" s="159" t="s">
+      <c r="FF6" s="121" t="s">
         <v>12</v>
       </c>
-      <c r="FG6" s="140"/>
-      <c r="FH6" s="140"/>
-      <c r="FI6" s="140"/>
+      <c r="FG6" s="134"/>
+      <c r="FH6" s="134"/>
+      <c r="FI6" s="134"/>
       <c r="FJ6" s="135"/>
       <c r="FK6" s="71"/>
-      <c r="FL6" s="121" t="s">
+      <c r="FL6" s="138" t="s">
         <v>108</v>
       </c>
-      <c r="FM6" s="122"/>
-      <c r="FN6" s="122"/>
-      <c r="FO6" s="123"/>
-      <c r="FP6" s="121" t="s">
+      <c r="FM6" s="139"/>
+      <c r="FN6" s="139"/>
+      <c r="FO6" s="140"/>
+      <c r="FP6" s="138" t="s">
         <v>118</v>
       </c>
-      <c r="FQ6" s="122"/>
-      <c r="FR6" s="122"/>
-      <c r="FS6" s="122"/>
-      <c r="FT6" s="122"/>
-      <c r="FU6" s="123"/>
+      <c r="FQ6" s="139"/>
+      <c r="FR6" s="139"/>
+      <c r="FS6" s="139"/>
+      <c r="FT6" s="139"/>
+      <c r="FU6" s="140"/>
       <c r="FV6" s="70"/>
-      <c r="FW6" s="133" t="s">
+      <c r="FW6" s="144" t="s">
         <v>13</v>
       </c>
-      <c r="FX6" s="164"/>
-      <c r="FY6" s="164"/>
-      <c r="FZ6" s="165"/>
-      <c r="GA6" s="169" t="s">
+      <c r="FX6" s="145"/>
+      <c r="FY6" s="145"/>
+      <c r="FZ6" s="146"/>
+      <c r="GA6" s="175" t="s">
         <v>14</v>
       </c>
-      <c r="GB6" s="121" t="s">
+      <c r="GB6" s="138" t="s">
         <v>15</v>
       </c>
-      <c r="GC6" s="122"/>
-      <c r="GD6" s="122"/>
-      <c r="GE6" s="123"/>
-      <c r="GF6" s="159" t="s">
+      <c r="GC6" s="139"/>
+      <c r="GD6" s="139"/>
+      <c r="GE6" s="140"/>
+      <c r="GF6" s="121" t="s">
         <v>16</v>
       </c>
-      <c r="GG6" s="171" t="s">
+      <c r="GG6" s="123" t="s">
         <v>17</v>
       </c>
-      <c r="GH6" s="173" t="s">
+      <c r="GH6" s="125" t="s">
         <v>11</v>
       </c>
-      <c r="GI6" s="152" t="s">
+      <c r="GI6" s="127" t="s">
         <v>10</v>
       </c>
-      <c r="GJ6" s="175" t="s">
+      <c r="GJ6" s="129" t="s">
         <v>9</v>
       </c>
       <c r="GK6" s="1"/>
@@ -9114,22 +9113,22 @@
       <c r="C7" s="21"/>
       <c r="D7" s="51"/>
       <c r="E7" s="51"/>
-      <c r="F7" s="130"/>
-      <c r="G7" s="131"/>
-      <c r="H7" s="131"/>
-      <c r="I7" s="131"/>
-      <c r="J7" s="131"/>
-      <c r="K7" s="131"/>
-      <c r="L7" s="131"/>
-      <c r="M7" s="131"/>
-      <c r="N7" s="131"/>
-      <c r="O7" s="131"/>
-      <c r="P7" s="131"/>
-      <c r="Q7" s="131"/>
-      <c r="R7" s="131"/>
-      <c r="S7" s="131"/>
-      <c r="T7" s="131"/>
-      <c r="U7" s="132"/>
+      <c r="F7" s="156"/>
+      <c r="G7" s="157"/>
+      <c r="H7" s="157"/>
+      <c r="I7" s="157"/>
+      <c r="J7" s="157"/>
+      <c r="K7" s="157"/>
+      <c r="L7" s="157"/>
+      <c r="M7" s="157"/>
+      <c r="N7" s="157"/>
+      <c r="O7" s="157"/>
+      <c r="P7" s="157"/>
+      <c r="Q7" s="157"/>
+      <c r="R7" s="157"/>
+      <c r="S7" s="157"/>
+      <c r="T7" s="157"/>
+      <c r="U7" s="158"/>
       <c r="V7" s="3"/>
       <c r="W7" s="51" t="s">
         <v>18</v>
@@ -9258,63 +9257,63 @@
       <c r="EC7" s="51"/>
       <c r="ED7" s="51"/>
       <c r="EE7" s="51"/>
-      <c r="EF7" s="136"/>
-      <c r="EG7" s="137"/>
-      <c r="EH7" s="137"/>
-      <c r="EI7" s="138"/>
+      <c r="EF7" s="160"/>
+      <c r="EG7" s="161"/>
+      <c r="EH7" s="161"/>
+      <c r="EI7" s="162"/>
       <c r="EJ7" s="68"/>
-      <c r="EK7" s="141"/>
-      <c r="EL7" s="142"/>
-      <c r="EM7" s="142"/>
-      <c r="EN7" s="142"/>
-      <c r="EO7" s="142"/>
-      <c r="EP7" s="142"/>
-      <c r="EQ7" s="146"/>
-      <c r="ER7" s="147"/>
-      <c r="ES7" s="148"/>
+      <c r="EK7" s="164"/>
+      <c r="EL7" s="136"/>
+      <c r="EM7" s="136"/>
+      <c r="EN7" s="136"/>
+      <c r="EO7" s="136"/>
+      <c r="EP7" s="136"/>
+      <c r="EQ7" s="168"/>
+      <c r="ER7" s="169"/>
+      <c r="ES7" s="170"/>
       <c r="ET7" s="67"/>
-      <c r="EU7" s="150"/>
-      <c r="EV7" s="151"/>
+      <c r="EU7" s="172"/>
+      <c r="EV7" s="137"/>
       <c r="EW7" s="67"/>
-      <c r="EX7" s="153"/>
+      <c r="EX7" s="128"/>
       <c r="EY7" s="67"/>
-      <c r="EZ7" s="155"/>
-      <c r="FA7" s="142"/>
-      <c r="FB7" s="142"/>
-      <c r="FC7" s="142"/>
-      <c r="FD7" s="151"/>
+      <c r="EZ7" s="174"/>
+      <c r="FA7" s="136"/>
+      <c r="FB7" s="136"/>
+      <c r="FC7" s="136"/>
+      <c r="FD7" s="137"/>
       <c r="FE7" s="67"/>
-      <c r="FF7" s="160"/>
-      <c r="FG7" s="142"/>
-      <c r="FH7" s="142"/>
-      <c r="FI7" s="142"/>
-      <c r="FJ7" s="151"/>
+      <c r="FF7" s="122"/>
+      <c r="FG7" s="136"/>
+      <c r="FH7" s="136"/>
+      <c r="FI7" s="136"/>
+      <c r="FJ7" s="137"/>
       <c r="FK7" s="67"/>
-      <c r="FL7" s="161"/>
-      <c r="FM7" s="162"/>
-      <c r="FN7" s="162"/>
-      <c r="FO7" s="163"/>
-      <c r="FP7" s="161"/>
-      <c r="FQ7" s="162"/>
-      <c r="FR7" s="162"/>
-      <c r="FS7" s="162"/>
-      <c r="FT7" s="162"/>
-      <c r="FU7" s="163"/>
+      <c r="FL7" s="141"/>
+      <c r="FM7" s="142"/>
+      <c r="FN7" s="142"/>
+      <c r="FO7" s="143"/>
+      <c r="FP7" s="141"/>
+      <c r="FQ7" s="142"/>
+      <c r="FR7" s="142"/>
+      <c r="FS7" s="142"/>
+      <c r="FT7" s="142"/>
+      <c r="FU7" s="143"/>
       <c r="FV7" s="51"/>
-      <c r="FW7" s="166"/>
-      <c r="FX7" s="167"/>
-      <c r="FY7" s="167"/>
-      <c r="FZ7" s="168"/>
-      <c r="GA7" s="170"/>
-      <c r="GB7" s="124"/>
-      <c r="GC7" s="125"/>
-      <c r="GD7" s="125"/>
-      <c r="GE7" s="126"/>
-      <c r="GF7" s="160"/>
-      <c r="GG7" s="172"/>
-      <c r="GH7" s="174"/>
-      <c r="GI7" s="153"/>
-      <c r="GJ7" s="176"/>
+      <c r="FW7" s="147"/>
+      <c r="FX7" s="148"/>
+      <c r="FY7" s="148"/>
+      <c r="FZ7" s="149"/>
+      <c r="GA7" s="176"/>
+      <c r="GB7" s="150"/>
+      <c r="GC7" s="151"/>
+      <c r="GD7" s="151"/>
+      <c r="GE7" s="152"/>
+      <c r="GF7" s="122"/>
+      <c r="GG7" s="124"/>
+      <c r="GH7" s="126"/>
+      <c r="GI7" s="128"/>
+      <c r="GJ7" s="130"/>
       <c r="GK7" s="1"/>
     </row>
     <row r="8" spans="1:193" ht="17" x14ac:dyDescent="0.4">
@@ -9914,7 +9913,7 @@
         <v>51.818549201858957</v>
       </c>
       <c r="X9" s="24">
-        <f t="shared" ref="X9:AH24" si="0">IF(K9="","",K9/SUM($J9:$U9)*100)</f>
+        <f t="shared" ref="X9:AG9" si="0">IF(K9="","",K9/SUM($J9:$U9)*100)</f>
         <v>2.5257627803596683</v>
       </c>
       <c r="Y9" s="24">
@@ -9971,7 +9970,7 @@
         <v>3.5624298735679377E-2</v>
       </c>
       <c r="AM9" s="47">
-        <f t="shared" ref="AM9:AM72" si="1">IF(Y9="","",Y9/101.96)</f>
+        <f t="shared" ref="AM9" si="1">IF(Y9="","",Y9/101.96)</f>
         <v>0.13575107921117088</v>
       </c>
       <c r="AN9" s="49">
@@ -9983,31 +9982,31 @@
         <v>0.18561771406337652</v>
       </c>
       <c r="AP9" s="47">
-        <f t="shared" ref="AP9:AP72" si="2">IF(AB9="","",AB9/71)</f>
+        <f t="shared" ref="AP9" si="2">IF(AB9="","",AB9/71)</f>
         <v>2.8459298933630067E-4</v>
       </c>
       <c r="AQ9" s="47">
-        <f t="shared" ref="AQ9:AQ72" si="3">IF(AC9="","",AC9/56.08)</f>
+        <f t="shared" ref="AQ9" si="3">IF(AC9="","",AC9/56.08)</f>
         <v>0.12070335683601841</v>
       </c>
       <c r="AR9" s="47">
-        <f t="shared" ref="AR9:AR72" si="4">IF(AD9="","",AD9/56.1)</f>
+        <f t="shared" ref="AR9" si="4">IF(AD9="","",AD9/56.1)</f>
         <v>0.19863931171028265</v>
       </c>
       <c r="AS9" s="47">
-        <f t="shared" ref="AS9:AS72" si="5">IF(AE9="","",AE9/62)</f>
+        <f t="shared" ref="AS9" si="5">IF(AE9="","",AE9/62)</f>
         <v>3.6990203299460948E-2</v>
       </c>
       <c r="AT9" s="47">
-        <f t="shared" ref="AT9:AT72" si="6">IF(AF9="","",AF9/94.2)</f>
+        <f t="shared" ref="AT9" si="6">IF(AF9="","",AF9/94.2)</f>
         <v>4.6117961594677589E-3</v>
       </c>
       <c r="AU9" s="47">
-        <f t="shared" ref="AU9:AU72" si="7">IF(AG9="","",AG9/70.97)</f>
+        <f t="shared" ref="AU9" si="7">IF(AG9="","",AG9/70.97)</f>
         <v>0</v>
       </c>
       <c r="AV9" s="47">
-        <f t="shared" ref="AV9:AV72" si="8">IF(AH9="","",AH9/18.02)</f>
+        <f t="shared" ref="AV9" si="8">IF(AH9="","",AH9/18.02)</f>
         <v>0</v>
       </c>
       <c r="AW9" s="47">
@@ -10015,11 +10014,11 @@
         <v>1.5805713162575632</v>
       </c>
       <c r="AX9" s="47">
-        <f t="shared" ref="AX9:AX72" si="9">IF(OR(AA9="",I9=""),"",$AA9*(1-$EP9)/71.85)</f>
+        <f t="shared" ref="AX9" si="9">IF(OR(AA9="",I9=""),"",$AA9*(1-$EP9)/71.85)</f>
         <v>0.13976680660567234</v>
       </c>
       <c r="AY9" s="46">
-        <f t="shared" ref="AY9:AY72" si="10">IF(OR(AA9="",I9=""),"",($AA9*$EP9)*1.111/159.6)</f>
+        <f t="shared" ref="AY9" si="10">IF(OR(AA9="",I9=""),"",($AA9*$EP9)*1.111/159.6)</f>
         <v>7.7374842043469423E-3</v>
       </c>
       <c r="AZ9" s="26"/>
@@ -10028,55 +10027,55 @@
         <v>0.54559320062483363</v>
       </c>
       <c r="BB9" s="44">
-        <f t="shared" ref="BB9:BB72" si="11">IF(OR(AW9="",$AL9=""),"",AL9/$AW9)</f>
+        <f t="shared" ref="BB9" si="11">IF(OR(AW9="",$AL9=""),"",AL9/$AW9)</f>
         <v>2.2538874626694915E-2</v>
       </c>
       <c r="BC9" s="44">
-        <f t="shared" ref="BC9:BC72" si="12">IF(OR(AW9="",$AM9=""),"",AM9/$AW9)</f>
+        <f t="shared" ref="BC9" si="12">IF(OR(AW9="",$AM9=""),"",AM9/$AW9)</f>
         <v>8.5887348337181549E-2</v>
       </c>
       <c r="BD9" s="44">
-        <f t="shared" ref="BD9:BD72" si="13">IF(OR(AW9="",$AN9=""),"",AN9/$AW9)</f>
+        <f t="shared" ref="BD9" si="13">IF(OR(AW9="",$AN9=""),"",AN9/$AW9)</f>
         <v>0</v>
       </c>
       <c r="BE9" s="44">
-        <f t="shared" ref="BE9:BE72" si="14">IF(OR(AW9="",$AO9=""),"",AO9/$AW9)</f>
+        <f t="shared" ref="BE9" si="14">IF(OR(AW9="",$AO9=""),"",AO9/$AW9)</f>
         <v>0.11743710147978483</v>
       </c>
       <c r="BF9" s="44">
-        <f t="shared" ref="BF9:BF72" si="15">IF(OR(AW9="",$AX9=""),"",AX9/$AW9)</f>
+        <f t="shared" ref="BF9" si="15">IF(OR(AW9="",$AX9=""),"",AX9/$AW9)</f>
         <v>8.842802926261413E-2</v>
       </c>
       <c r="BG9" s="44">
-        <f t="shared" ref="BG9:BG72" si="16">IF(OR(AW9="",$AY9=""),"",AY9/$AW9)</f>
+        <f t="shared" ref="BG9" si="16">IF(OR(AW9="",$AY9=""),"",AY9/$AW9)</f>
         <v>4.8953717714348768E-3</v>
       </c>
       <c r="BH9" s="44">
-        <f t="shared" ref="BH9:BH72" si="17">IF(OR(AW9="",$AP9=""),"",AP9/$AW9)</f>
+        <f t="shared" ref="BH9" si="17">IF(OR(AW9="",$AP9=""),"",AP9/$AW9)</f>
         <v>1.8005703786283606E-4</v>
       </c>
       <c r="BI9" s="44">
-        <f t="shared" ref="BI9:BI72" si="18">IF(OR(AW9="",$AQ9=""),"",AQ9/$AW9)</f>
+        <f t="shared" ref="BI9" si="18">IF(OR(AW9="",$AQ9=""),"",AQ9/$AW9)</f>
         <v>7.6366915933800919E-2</v>
       </c>
       <c r="BJ9" s="44">
-        <f t="shared" ref="BJ9:BJ72" si="19">IF(OR(AW9="",$AR9=""),"",AR9/$AW9)</f>
+        <f t="shared" ref="BJ9" si="19">IF(OR(AW9="",$AR9=""),"",AR9/$AW9)</f>
         <v>0.1256756399835319</v>
       </c>
       <c r="BK9" s="44">
-        <f t="shared" ref="BK9:BK72" si="20">IF(OR(AW9="",$AS9=""),"",AS9/$AW9)</f>
+        <f t="shared" ref="BK9" si="20">IF(OR(AW9="",$AS9=""),"",AS9/$AW9)</f>
         <v>2.3403058703510712E-2</v>
       </c>
       <c r="BL9" s="44">
-        <f t="shared" ref="BL9:BL72" si="21">IF(OR(AW9="",$AT9=""),"",AT9/$AW9)</f>
+        <f t="shared" ref="BL9" si="21">IF(OR(AW9="",$AT9=""),"",AT9/$AW9)</f>
         <v>2.9178032727985052E-3</v>
       </c>
       <c r="BM9" s="44">
-        <f t="shared" ref="BM9:BM72" si="22">IF(OR(AW9="",$AU9=""),"",AU9/$AW9)</f>
+        <f t="shared" ref="BM9" si="22">IF(OR(AW9="",$AU9=""),"",AU9/$AW9)</f>
         <v>0</v>
       </c>
       <c r="BN9" s="44">
-        <f t="shared" ref="BN9:BN72" si="23">IF(OR(AV9="",AW9=""),"",AV9/AW9)</f>
+        <f t="shared" ref="BN9" si="23">IF(OR(AV9="",AW9=""),"",AV9/AW9)</f>
         <v>0</v>
       </c>
       <c r="BO9" s="43">
@@ -10089,64 +10088,64 @@
         <v>1.7246979265055402</v>
       </c>
       <c r="BR9" s="44">
-        <f t="shared" ref="BR9:BR72" si="24">IF(X9="","",X9/(79.9/2))</f>
+        <f t="shared" ref="BR9" si="24">IF(X9="","",X9/(79.9/2))</f>
         <v>6.322309838196917E-2</v>
       </c>
       <c r="BS9" s="44">
-        <f t="shared" ref="BS9:BS72" si="25">IF(Y9="","",Y9/(102/3))</f>
+        <f t="shared" ref="BS9" si="25">IF(Y9="","",Y9/(102/3))</f>
         <v>0.40709353048149949</v>
       </c>
       <c r="BT9" s="44">
-        <f t="shared" ref="BT9:BT72" si="26">IF(Z9="","",Z9/(151.9922/3))</f>
+        <f t="shared" ref="BT9" si="26">IF(Z9="","",Z9/(151.9922/3))</f>
         <v>0</v>
       </c>
       <c r="BU9" s="44">
-        <f t="shared" ref="BU9:BU72" si="27">IF(AA9="","",AA9/(71.85))</f>
+        <f t="shared" ref="BU9" si="27">IF(AA9="","",AA9/(71.85))</f>
         <v>0.15523686065509112</v>
       </c>
       <c r="BV9" s="13">
-        <f t="shared" ref="BV9:BV72" si="28">IF($AA9="","",$AA9*(1-$EP9)/71.85)</f>
+        <f t="shared" ref="BV9" si="28">IF($AA9="","",$AA9*(1-$EP9)/71.85)</f>
         <v>0.13976680660567234</v>
       </c>
       <c r="BW9" s="24">
-        <f t="shared" ref="BW9:BW72" si="29">IF(AA9="","",$AA9*$EP9*1.111/(159.6/3))</f>
+        <f t="shared" ref="BW9" si="29">IF(AA9="","",$AA9*$EP9*1.111/(159.6/3))</f>
         <v>2.3212452613040828E-2</v>
       </c>
       <c r="BX9" s="44">
-        <f t="shared" ref="BX9:BX72" si="30">IF(AB9="","",AB9/71)</f>
+        <f t="shared" ref="BX9" si="30">IF(AB9="","",AB9/71)</f>
         <v>2.8459298933630067E-4</v>
       </c>
       <c r="BY9" s="44">
-        <f t="shared" ref="BY9:BY72" si="31">IF(AC9="","",AC9/40.3)</f>
+        <f t="shared" ref="BY9" si="31">IF(AC9="","",AC9/40.3)</f>
         <v>0.16796635859463802</v>
       </c>
       <c r="BZ9" s="44">
-        <f t="shared" ref="BZ9:BZ72" si="32">IF(AD9="","",AD9/56.1)</f>
+        <f t="shared" ref="BZ9" si="32">IF(AD9="","",AD9/56.1)</f>
         <v>0.19863931171028265</v>
       </c>
       <c r="CA9" s="44">
-        <f t="shared" ref="CA9:CA72" si="33">IF(AE9="","",AE9/62)</f>
+        <f t="shared" ref="CA9" si="33">IF(AE9="","",AE9/62)</f>
         <v>3.6990203299460948E-2</v>
       </c>
       <c r="CB9" s="44">
-        <f t="shared" ref="CB9:CB72" si="34">IF(AF9="","",AF9/94.2)</f>
+        <f t="shared" ref="CB9" si="34">IF(AF9="","",AF9/94.2)</f>
         <v>4.6117961594677589E-3</v>
       </c>
       <c r="CC9" s="44">
-        <f t="shared" ref="CC9:CC72" si="35">IF(AG9="","",AG9/(70.97/5))</f>
+        <f t="shared" ref="CC9" si="35">IF(AG9="","",AG9/(70.97/5))</f>
         <v>0</v>
       </c>
       <c r="CD9" s="44">
-        <f t="shared" ref="CD9:CD72" si="36">IF(AH9="","",AH9/(18.02))</f>
+        <f t="shared" ref="CD9" si="36">IF(AH9="","",AH9/(18.02))</f>
         <v>0</v>
       </c>
       <c r="CE9" s="12">
-        <f t="shared" ref="CE9:CE72" si="37">IF(SUM(BQ9:BU9,BX9:CD9)=0,"",SUM(BQ9:BU9,BX9:CD9))</f>
+        <f t="shared" ref="CE9" si="37">IF(SUM(BQ9:BU9,BX9:CD9)=0,"",SUM(BQ9:BU9,BX9:CD9))</f>
         <v>2.7587436787772859</v>
       </c>
       <c r="CF9" s="13"/>
       <c r="CG9" s="45">
-        <f t="shared" ref="CG9:CT27" si="38">IF(OR($CE9="",BQ9=""),"",BQ9/$CE9)</f>
+        <f t="shared" ref="CG9:CS9" si="38">IF(OR($CE9="",BQ9=""),"",BQ9/$CE9)</f>
         <v>0.6251751258275472</v>
       </c>
       <c r="CH9" s="44">
@@ -10202,60 +10201,60 @@
         <v>0</v>
       </c>
       <c r="CU9" s="12">
-        <f t="shared" ref="CU9:CU72" si="39">IF(SUM(CG9:CK9,CN9:CT9)=0,"",SUM(CG9:CK9,CN9:CT9))</f>
+        <f t="shared" ref="CU9" si="39">IF(SUM(CG9:CK9,CN9:CT9)=0,"",SUM(CG9:CK9,CN9:CT9))</f>
         <v>0.99999999999999989</v>
       </c>
       <c r="CV9" s="13"/>
       <c r="CW9" s="45">
-        <f t="shared" ref="CW9:CW72" si="40">IF(W9="","",W9/60.09)</f>
+        <f t="shared" ref="CW9" si="40">IF(W9="","",W9/60.09)</f>
         <v>0.86234896325277011</v>
       </c>
       <c r="CX9" s="44">
-        <f t="shared" ref="CX9:CX72" si="41">IF(X9="","",X9/79.9)</f>
+        <f t="shared" ref="CX9" si="41">IF(X9="","",X9/79.9)</f>
         <v>3.1611549190984585E-2</v>
       </c>
       <c r="CY9" s="44">
-        <f t="shared" ref="CY9:CY72" si="42">IF(Y9="","",Y9/(102/2))</f>
+        <f t="shared" ref="CY9" si="42">IF(Y9="","",Y9/(102/2))</f>
         <v>0.27139568698766631</v>
       </c>
       <c r="CZ9" s="44">
-        <f t="shared" ref="CZ9:CZ72" si="43">IF(Z9="","",Z9/(151.9922/2))</f>
+        <f t="shared" ref="CZ9" si="43">IF(Z9="","",Z9/(151.9922/2))</f>
         <v>0</v>
       </c>
       <c r="DA9" s="44">
-        <f t="shared" ref="DA9:DA72" si="44">IF(Q9="","",Q9/71.8)</f>
+        <f t="shared" ref="DA9" si="44">IF(Q9="","",Q9/71.8)</f>
         <v>0.15362116991643454</v>
       </c>
       <c r="DB9" s="44">
-        <f t="shared" ref="DB9:DB72" si="45">IF($AA9="","",$AA9*(1-$EP9)/71.85)</f>
+        <f>IF($AA9="","",$AA9*(1-$EP9)/71.85)</f>
         <v>0.13976680660567234</v>
       </c>
       <c r="DC9" s="47">
-        <f t="shared" ref="DC9:DC72" si="46">IF($AA9="","",$AA9*$EP9*1.111/(159.6/2))</f>
+        <f t="shared" ref="DC9" si="45">IF($AA9="","",$AA9*$EP9*1.111/(159.6/2))</f>
         <v>1.5474968408693885E-2</v>
       </c>
       <c r="DD9" s="44">
-        <f t="shared" ref="DD9:DD72" si="47">IF(AB9="","",AB9/71)</f>
+        <f t="shared" ref="DD9" si="46">IF(AB9="","",AB9/71)</f>
         <v>2.8459298933630067E-4</v>
       </c>
       <c r="DE9" s="44">
-        <f t="shared" ref="DE9:DE72" si="48">IF(AC9="","",AC9/40.3)</f>
+        <f t="shared" ref="DE9" si="47">IF(AC9="","",AC9/40.3)</f>
         <v>0.16796635859463802</v>
       </c>
       <c r="DF9" s="44">
-        <f t="shared" ref="DF9:DF72" si="49">IF(AD9="","",AD9/56.1)</f>
+        <f t="shared" ref="DF9" si="48">IF(AD9="","",AD9/56.1)</f>
         <v>0.19863931171028265</v>
       </c>
       <c r="DG9" s="44">
-        <f t="shared" ref="DG9:DG72" si="50">IF(AE9="","",AE9/(62/2))</f>
+        <f t="shared" ref="DG9" si="49">IF(AE9="","",AE9/(62/2))</f>
         <v>7.3980406598921897E-2</v>
       </c>
       <c r="DH9" s="44">
-        <f t="shared" ref="DH9:DH72" si="51">IF(AF9="","",AF9/(94.2/2))</f>
+        <f t="shared" ref="DH9" si="50">IF(AF9="","",AF9/(94.2/2))</f>
         <v>9.2235923189355178E-3</v>
       </c>
       <c r="DI9" s="44">
-        <f t="shared" ref="DI9:DI72" si="52">IF(AG9="","",AG9/(70.97/2))</f>
+        <f t="shared" ref="DI9" si="51">IF(AG9="","",AG9/(70.97/2))</f>
         <v>0</v>
       </c>
       <c r="DJ9" s="44">
@@ -10272,68 +10271,68 @@
         <v>0.48745847701619049</v>
       </c>
       <c r="DN9" s="44">
-        <f t="shared" ref="DN9:DZ24" si="53">IF(OR($DK9="",CX9=""),"",CX9/$DK9)</f>
+        <f t="shared" ref="DN9:DZ9" si="52">IF(OR($DK9="",CX9=""),"",CX9/$DK9)</f>
         <v>1.7869004638952624E-2</v>
       </c>
       <c r="DO9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>0.15341136116028792</v>
       </c>
       <c r="DP9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>0</v>
       </c>
       <c r="DQ9" s="44">
-        <f t="shared" si="53"/>
+        <f>IF(OR($DK9="",DA9=""),"",DA9/$DK9)</f>
         <v>8.6837167684934949E-2</v>
       </c>
       <c r="DR9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>7.9005736179504377E-2</v>
       </c>
       <c r="DS9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>8.7475080899059119E-3</v>
       </c>
       <c r="DT9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>1.6087137697490868E-4</v>
       </c>
       <c r="DU9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>9.4946047179856163E-2</v>
       </c>
       <c r="DV9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>0.11228449327126581</v>
       </c>
       <c r="DW9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>4.1818773914590372E-2</v>
       </c>
       <c r="DX9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>5.2138037569468805E-3</v>
       </c>
       <c r="DY9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>0</v>
       </c>
       <c r="DZ9" s="44">
-        <f t="shared" si="53"/>
+        <f t="shared" si="52"/>
         <v>0</v>
       </c>
       <c r="EA9" s="43">
-        <f t="shared" ref="EA9:EA72" si="54">IF($DK9="","",DK9/$DK9)</f>
+        <f t="shared" ref="EA9" si="53">IF($DK9="","",DK9/$DK9)</f>
         <v>1</v>
       </c>
       <c r="EB9" s="26"/>
       <c r="EC9" s="30">
-        <f t="shared" ref="EC9:EC72" si="55">IF(G9="","",G9+273)</f>
+        <f t="shared" ref="EC9" si="54">IF(G9="","",G9+273)</f>
         <v>1473</v>
       </c>
       <c r="ED9" s="14">
-        <f t="shared" ref="ED9:ED72" si="56">IF(H9="","",H9*1000000000)</f>
+        <f t="shared" ref="ED9" si="55">IF(H9="","",H9*1000000000)</f>
         <v>10000000</v>
       </c>
       <c r="EE9" s="29"/>
@@ -10350,16 +10349,16 @@
         <v>-1.7336286490156159</v>
       </c>
       <c r="EI9" s="12">
-        <f t="shared" ref="EI9:EI72" si="57">IF(EF9="","",27489/($EC9)-6.702-0.055*($ED9/100000)/($EC9)+$EF9)</f>
+        <f t="shared" ref="EI9" si="56">IF(EF9="","",27489/($EC9)-6.702-0.055*($ED9/100000)/($EC9)+$EF9)</f>
         <v>2.6610312287847915</v>
       </c>
       <c r="EJ9" s="29"/>
       <c r="EK9" s="28">
-        <f t="shared" ref="EK9:EK72" si="58">IF(OR(EF9="",AW9=""),"",0.196*LN(10^$EF9)+11492/$EC9-6.675+($BC9*-2.243+$BE9*-1.828+$BJ9*3.201+$BK9*5.854+$BL9*6.215)-3.36*(1-1673/$EC9-LN($EC9/1673))-0.000000701*($ED9/$EC9)-0.000000000154*(($EC9-1673)*$ED9/$EC9)+0.0000000000000000385*($ED9^2/$EC9))</f>
+        <f t="shared" ref="EK9" si="57">IF(OR(EF9="",AW9=""),"",0.196*LN(10^$EF9)+11492/$EC9-6.675+($BC9*-2.243+$BE9*-1.828+$BJ9*3.201+$BK9*5.854+$BL9*6.215)-3.36*(1-1673/$EC9-LN($EC9/1673))-0.000000701*($ED9/$EC9)-0.000000000154*(($EC9-1673)*$ED9/$EC9)+0.0000000000000000385*($ED9^2/$EC9))</f>
         <v>-2.8942163889007162</v>
       </c>
       <c r="EL9" s="24">
-        <f t="shared" ref="EL9:EL72" si="59">IF(EK9="","",EK9/2.303)</f>
+        <f t="shared" ref="EL9" si="58">IF(EK9="","",EK9/2.303)</f>
         <v>-1.2567157572300114</v>
       </c>
       <c r="EM9" s="24">
@@ -10367,27 +10366,27 @@
         <v>5.5342375007053163E-2</v>
       </c>
       <c r="EN9" s="24">
-        <f t="shared" ref="EN9:EN72" si="60">IF(OR(AA9=0,EM9=""),"",BE9/(1+2*EM9))</f>
+        <f t="shared" ref="EN9" si="59">IF(OR(AA9=0,EM9=""),"",BE9/(1+2*EM9))</f>
         <v>0.10573396409583664</v>
       </c>
       <c r="EO9" s="24">
-        <f t="shared" ref="EO9:EO72" si="61">IF(OR(AA9=0,EM9=""),"",EM9*EN9)</f>
+        <f t="shared" ref="EO9" si="60">IF(OR(AA9=0,EM9=""),"",EM9*EN9)</f>
         <v>5.8515686919740862E-3</v>
       </c>
       <c r="EP9" s="24">
-        <f t="shared" ref="EP9:EP72" si="62">IF(EN9="","",EO9*2/(EO9*2+EN9))</f>
+        <f t="shared" ref="EP9" si="61">IF(EN9="","",EO9*2/(EO9*2+EN9))</f>
         <v>9.9654514940175937E-2</v>
       </c>
       <c r="EQ9" s="24">
-        <f t="shared" ref="EQ9:EQ72" si="63">IF(AA9="","",LN(AY9/AX9))</f>
+        <f t="shared" ref="EQ9" si="62">IF(AA9="","",LN(AY9/AX9))</f>
         <v>-2.8938987701739523</v>
       </c>
       <c r="ER9" s="24">
-        <f t="shared" ref="ER9:ER72" si="64">IF(EQ9="","",(11492/$EC9-6.675+($BC9*-2.243+$BE9*-1.828+$BJ9*3.201+$BK9*5.854+$BL9*6.215)-3.36*(1-1673/$EC9-LN($EC9/1673))-0.000000701*($ED9/$EC9)-0.000000000154*(($EC9-1673)*$ED9/$EC9)+0.0000000000000000385*($ED9^2/$EC9)-$EQ9)/-0.196)</f>
+        <f t="shared" ref="ER9" si="63">IF(EQ9="","",(11492/$EC9-6.675+($BC9*-2.243+$BE9*-1.828+$BJ9*3.201+$BK9*5.854+$BL9*6.215)-3.36*(1-1673/$EC9-LN($EC9/1673))-0.000000701*($ED9/$EC9)-0.000000000154*(($EC9-1673)*$ED9/$EC9)+0.0000000000000000385*($ED9^2/$EC9)-$EQ9)/-0.196)</f>
         <v>-21.401251838401116</v>
       </c>
       <c r="ES9" s="25">
-        <f t="shared" ref="ES9:ES72" si="65">IF(ER9="","",ER9/2.303)</f>
+        <f t="shared" ref="ES9" si="64">IF(ER9="","",ER9/2.303)</f>
         <v>-9.2927710978728246</v>
       </c>
       <c r="ET9" s="26"/>
@@ -10396,7 +10395,7 @@
         <v>-4.5588183168215686</v>
       </c>
       <c r="EV9" s="43">
-        <f t="shared" ref="EV9:EV72" si="66">IF(EU9="","",1-1/(1+10^EU9))</f>
+        <f t="shared" ref="EV9" si="65">IF(EU9="","",1-1/(1+10^EU9))</f>
         <v>2.7616566910748652E-5</v>
       </c>
       <c r="EW9" s="26"/>
@@ -10406,73 +10405,73 @@
       </c>
       <c r="EY9" s="26"/>
       <c r="EZ9" s="45">
-        <f t="shared" ref="EZ9:EZ40" si="67">IF(EA9="","",-23590/(EC9)+8.77+(1673/(EC9))*(6.7*(DW9+DX9)+1.8*DO9+4.9*DU9+8.1*DV9+5*DN9+8.9*(DQ9+DT9)-22.2*(DQ9+DT9)*DN9+7.2*(DQ9+DT9)*DM9)-2.06*ERF(-7.2*DQ9+DT9))</f>
+        <f t="shared" ref="EZ9" si="66">IF(EA9="","",-23590/(EC9)+8.77+(1673/(EC9))*(6.7*(DW9+DX9)+1.8*DO9+4.9*DU9+8.1*DV9+5*DN9+8.9*(DQ9+DT9)-22.2*(DQ9+DT9)*DN9+7.2*(DQ9+DT9)*DM9)-2.06*ERF(-7.2*DQ9+DT9))</f>
         <v>-2.4395312413693455</v>
       </c>
       <c r="FA9" s="44">
-        <f t="shared" ref="FA9:FA72" si="68">IF($EA9="","",-8.02+(21100+44000*$DW9+18700*$DU9+4300*$DO9+44200*$DX9+35600*$DV9+12600*$DT9+16500*$DR9)/($EC9))</f>
+        <f t="shared" ref="FA9" si="67">IF($EA9="","",-8.02+(21100+44000*$DW9+18700*$DU9+4300*$DO9+44200*$DX9+35600*$DV9+12600*$DT9+16500*$DR9)/($EC9))</f>
         <v>12.963425458465952</v>
       </c>
       <c r="FB9" s="44">
-        <f t="shared" ref="FB9:FB40" si="69">IF(G9="","",-55921/(EC9)+25.07-0.6465*LN(EC9))</f>
+        <f t="shared" ref="FB9" si="68">IF(G9="","",-55921/(EC9)+25.07-0.6465*LN(EC9))</f>
         <v>-17.610272982068615</v>
       </c>
       <c r="FC9" s="13">
-        <f t="shared" ref="FC9:FC40" si="70">IF(EZ9="","",(FA9-FB9-EZ9)+2*LN(10)*EF9)</f>
+        <f t="shared" ref="FC9" si="69">IF(EZ9="","",(FA9-FB9-EZ9)+2*LN(10)*EF9)</f>
         <v>-9.7925150023142749</v>
       </c>
       <c r="FD9" s="43">
-        <f t="shared" ref="FD9:FD72" si="71">IF(FC9="","",1-1/(1+EXP(FC9)))</f>
+        <f t="shared" ref="FD9" si="70">IF(FC9="","",1-1/(1+EXP(FC9)))</f>
         <v>5.5865090669016126E-5</v>
       </c>
       <c r="FE9" s="13"/>
       <c r="FF9" s="45">
-        <f t="shared" ref="FF9:FF40" si="72">IF(CU9="","",0.225+(25237*CL9+5214*CP9+12705*CN9+19829*CR9-1109*CG9-8879)/(EC9))</f>
+        <f t="shared" ref="FF9" si="71">IF(CU9="","",0.225+(25237*CL9+5214*CP9+12705*CN9+19829*CR9-1109*CG9-8879)/(EC9))</f>
         <v>-5.127237973999927</v>
       </c>
       <c r="FG9" s="44">
-        <f t="shared" ref="FG9:FG40" si="73">IF(CU9="","",-12.948+(28649*CQ9+15602*CP9+9496*CO9+16016*CN9+4194*CI9+29244)/(EC9))</f>
+        <f t="shared" ref="FG9" si="72">IF(CU9="","",-12.948+(28649*CQ9+15602*CP9+9496*CO9+16016*CN9+4194*CI9+29244)/(EC9))</f>
         <v>8.7425899501378659</v>
       </c>
       <c r="FH9" s="44">
-        <f t="shared" ref="FH9:FH40" si="74">IF(CU9="","",-213.65+(25696*CQ9+15076*CP9+9543*CO9+16158*CN9+4316*CI9+68254)/(EC9)+55.03*LOG(EC9))</f>
+        <f t="shared" ref="FH9" si="73">IF(CU9="","",-213.65+(25696*CQ9+15076*CP9+9543*CO9+16158*CN9+4316*CI9+68254)/(EC9)+55.03*LOG(EC9))</f>
         <v>8.8317364872643225</v>
       </c>
       <c r="FI9" s="47">
-        <f t="shared" ref="FI9:FI40" si="75">IF(FF9="","",1-1/(1+10^(FG9-$FF9+2*$EF9)))</f>
+        <f t="shared" ref="FI9" si="74">IF(FF9="","",1-1/(1+10^(FG9-$FF9+2*$EF9)))</f>
         <v>1.9033600419993135E-5</v>
       </c>
       <c r="FJ9" s="46">
-        <f t="shared" ref="FJ9:FJ40" si="76">IF(FH9="","",1-1/(1+10^(FH9-$FF9+2*$EF9)))</f>
+        <f t="shared" ref="FJ9" si="75">IF(FH9="","",1-1/(1+10^(FH9-$FF9+2*$EF9)))</f>
         <v>2.3370370710540378E-5</v>
       </c>
       <c r="FK9" s="13"/>
       <c r="FL9" s="23">
-        <f t="shared" ref="FL9:FL72" si="77">IF($CU9="","",195.99657+(-7632.6971*$CG9-10669.7107*$CH9-6900.9065*$CI9-4625.0612*$CK9+19113.53*$CN9+11739.931*$CP9+33266.912*$CQ9-4094.9829)/$EC9-57.2083*LOG($EC9))</f>
+        <f>IF($CU9="","",195.99657+(-7632.6971*$CG9-10669.7107*$CH9-6900.9065*$CI9-4625.0612*$CK9+19113.53*$CN9+11739.931*$CP9+33266.912*$CQ9-4094.9829)/$EC9-57.2083*LOG($EC9))</f>
         <v>8.57357021121868</v>
       </c>
       <c r="FM9" s="13">
-        <f t="shared" ref="FM9:FM72" si="78">IF($CU9="","",0.646657+(-3368.52*$CG9-1233.439*$CI9+1295.54*$CP9+44885.3*$CR9+10914.48*($CG9*$CL9)-225569.4*($CL9*$CQ9)-871863.8*($CL9*$CR9)+54392.37*($CL9*$CI9)-7584.703)/($EC9)+3.86057*ERF($CL9))</f>
+        <f>IF($CU9="","",0.646657+(-3368.52*$CG9-1233.439*$CI9+1295.54*$CP9+44885.3*$CR9+10914.48*($CG9*$CL9)-225569.4*($CL9*$CQ9)-871863.8*($CL9*$CR9)+54392.37*($CL9*$CI9)-7584.703)/($EC9)+3.86057*ERF($CL9))</f>
         <v>-5.3643629299394</v>
       </c>
       <c r="FN9" s="13">
-        <f t="shared" ref="FN9:FN40" si="79">IF($FL9="","",$FL9-$FM9+2*$EF9)</f>
+        <f t="shared" ref="FN9" si="76">IF($FL9="","",$FL9-$FM9+2*$EF9)</f>
         <v>-4.6523655689573324</v>
       </c>
       <c r="FO9" s="13">
-        <f t="shared" ref="FO9:FO72" si="80">IF($FN9="","",1-1/(1+10^FN9))</f>
+        <f t="shared" ref="FO9" si="77">IF($FN9="","",1-1/(1+10^FN9))</f>
         <v>2.2265105705465693E-5</v>
       </c>
       <c r="FP9" s="23">
-        <f t="shared" ref="FP9:FP40" si="81">IF($FL9="","",$FL9-$FM9+2*($EF9-(0.0546*($H9*10000)/($G9+273))))</f>
+        <f>IF($FL9="","",$FL9-$FM9+2*($EF9-(0.0546*($H9*10000)/($G9+273))))</f>
         <v>-4.6597790109125263</v>
       </c>
       <c r="FQ9" s="13">
-        <f t="shared" ref="FQ9:FQ40" si="82">IF($FP9="","",1-1/(1+10^FP9))</f>
+        <f t="shared" ref="FQ9" si="78">IF($FP9="","",1-1/(1+10^FP9))</f>
         <v>2.1888272306647139E-5</v>
       </c>
       <c r="FR9" s="13">
-        <f t="shared" ref="FR9:FR40" si="83">IF($FL9="","",$FL9-$FM9+2*($EF9-(0.0332*($H9*10000)/($G9+273))))</f>
+        <f t="shared" ref="FR9" si="79">IF($FL9="","",$FL9-$FM9+2*($EF9-(0.0332*($H9*10000)/($G9+273))))</f>
         <v>-4.6568733761535306</v>
       </c>
       <c r="FS9" s="13">
@@ -10480,7 +10479,7 @@
         <v>2.2035202906667273E-5</v>
       </c>
       <c r="FT9" s="13">
-        <f t="shared" ref="FT9:FT40" si="84">IF($FL9="","",$FL9-$FM9+2*($EF9-(0.0601*($H9*10000)/($G9+273))))</f>
+        <f t="shared" ref="FT9" si="80">IF($FL9="","",$FL9-$FM9+2*($EF9-(0.0601*($H9*10000)/($G9+273))))</f>
         <v>-4.6605257862010525</v>
       </c>
       <c r="FU9" s="12">
@@ -10489,23 +10488,23 @@
       </c>
       <c r="FV9" s="22"/>
       <c r="FW9" s="42">
-        <f t="shared" ref="FW9:FW40" si="85">EG9</f>
+        <f t="shared" ref="FW9" si="81">EG9</f>
         <v>-1</v>
       </c>
       <c r="FX9" s="41">
-        <f t="shared" ref="FX9:FX40" si="86">EH9</f>
+        <f t="shared" ref="FX9" si="82">EH9</f>
         <v>-1.7336286490156159</v>
       </c>
       <c r="FY9" s="41">
-        <f t="shared" ref="FY9:FY40" si="87">EI9</f>
+        <f t="shared" ref="FY9" si="83">EI9</f>
         <v>2.6610312287847915</v>
       </c>
       <c r="FZ9" s="36">
-        <f t="shared" ref="FZ9:FZ40" si="88">EF9</f>
+        <f t="shared" ref="FZ9" si="84">EF9</f>
         <v>-9.2951493550577062</v>
       </c>
       <c r="GA9" s="10">
-        <f t="shared" ref="GA9:GA40" si="89">EP9</f>
+        <f t="shared" ref="GA9" si="85">EP9</f>
         <v>9.9654514940175937E-2</v>
       </c>
       <c r="GB9" s="40">
@@ -10525,23 +10524,23 @@
         <v>2.1888272306647139E-5</v>
       </c>
       <c r="GF9" s="37">
-        <f t="shared" ref="GF9:GF40" si="90">FI9</f>
+        <f t="shared" ref="GF9" si="86">FI9</f>
         <v>1.9033600419993135E-5</v>
       </c>
       <c r="GG9" s="36">
-        <f t="shared" ref="GG9:GG40" si="91">FJ9</f>
+        <f t="shared" ref="GG9" si="87">FJ9</f>
         <v>2.3370370710540378E-5</v>
       </c>
       <c r="GH9" s="35">
-        <f t="shared" ref="GH9:GH40" si="92">FD9</f>
+        <f t="shared" ref="GH9" si="88">FD9</f>
         <v>5.5865090669016126E-5</v>
       </c>
       <c r="GI9" s="35">
-        <f t="shared" ref="GI9:GI40" si="93">EX9</f>
+        <f t="shared" ref="GI9" si="89">EX9</f>
         <v>7.9426514400130776E-5</v>
       </c>
       <c r="GJ9" s="35">
-        <f t="shared" ref="GJ9:GJ40" si="94">EV9</f>
+        <f t="shared" ref="GJ9" si="90">EV9</f>
         <v>2.7616566910748652E-5</v>
       </c>
       <c r="GK9" s="1"/>
@@ -32007,16 +32006,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="GF6:GF7"/>
-    <mergeCell ref="GG6:GG7"/>
-    <mergeCell ref="GH6:GH7"/>
-    <mergeCell ref="GI6:GI7"/>
-    <mergeCell ref="GJ6:GJ7"/>
-    <mergeCell ref="U2:FW2"/>
-    <mergeCell ref="FF6:FJ7"/>
-    <mergeCell ref="FL6:FO7"/>
-    <mergeCell ref="FP6:FU7"/>
-    <mergeCell ref="FW6:FZ7"/>
     <mergeCell ref="GB6:GE7"/>
     <mergeCell ref="F6:U7"/>
     <mergeCell ref="EF6:EI7"/>
@@ -32026,8 +32015,24 @@
     <mergeCell ref="EX6:EX7"/>
     <mergeCell ref="EZ6:FD7"/>
     <mergeCell ref="GA6:GA7"/>
+    <mergeCell ref="U2:FW2"/>
+    <mergeCell ref="FF6:FJ7"/>
+    <mergeCell ref="FL6:FO7"/>
+    <mergeCell ref="FP6:FU7"/>
+    <mergeCell ref="FW6:FZ7"/>
+    <mergeCell ref="GF6:GF7"/>
+    <mergeCell ref="GG6:GG7"/>
+    <mergeCell ref="GH6:GH7"/>
+    <mergeCell ref="GI6:GI7"/>
+    <mergeCell ref="GJ6:GJ7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{1faf88fe-a998-4c5b-93c9-210a11d9a5c2}" enabled="0" method="" siteId="{1faf88fe-a998-4c5b-93c9-210a11d9a5c2}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>